<commit_message>
Update constraints: צרפתי limited to Sun night + Tue morning, עומר fixed Fri night
- צרפתי: only available Sun night + Tue morning (צו closes Tue night)
- עומר: fixed assignment Friday night
- External sheet: fill Wed evening gap with עומר

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/משמרות_29.3-4.4_v2.xlsx
+++ b/משמרות_29.3-4.4_v2.xlsx
@@ -102,14 +102,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFC000"/>
-        <bgColor rgb="00FFC000"/>
+        <fgColor rgb="00FFFF00"/>
+        <bgColor rgb="00FFFF00"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFF00"/>
-        <bgColor rgb="00FFFF00"/>
+        <fgColor rgb="00FFC000"/>
+        <bgColor rgb="00FFC000"/>
       </patternFill>
     </fill>
     <fill>
@@ -181,10 +181,10 @@
     <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -639,29 +639,29 @@
           <t>עומרי</t>
         </is>
       </c>
-      <c r="D2" s="5" t="inlineStr">
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>צרפתי</t>
+        </is>
+      </c>
+      <c r="E2" s="8" t="inlineStr">
+        <is>
+          <t>עומר</t>
+        </is>
+      </c>
+      <c r="F2" s="8" t="inlineStr">
+        <is>
+          <t>עומר</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
         <is>
           <t>ניר</t>
         </is>
       </c>
-      <c r="E2" s="7" t="inlineStr">
+      <c r="H2" s="8" t="inlineStr">
         <is>
           <t>עומר</t>
-        </is>
-      </c>
-      <c r="F2" s="8" t="inlineStr">
-        <is>
-          <t>צרפתי</t>
-        </is>
-      </c>
-      <c r="G2" s="7" t="inlineStr">
-        <is>
-          <t>עומר</t>
-        </is>
-      </c>
-      <c r="H2" s="9" t="inlineStr">
-        <is>
-          <t>משה</t>
         </is>
       </c>
     </row>
@@ -677,7 +677,7 @@
           <t>עומרי</t>
         </is>
       </c>
-      <c r="C3" s="7" t="inlineStr">
+      <c r="C3" s="8" t="inlineStr">
         <is>
           <t>עומר</t>
         </is>
@@ -689,7 +689,7 @@
       </c>
       <c r="E3" s="8" t="inlineStr">
         <is>
-          <t>צרפתי</t>
+          <t>עומר</t>
         </is>
       </c>
       <c r="F3" s="6" t="inlineStr">
@@ -715,7 +715,7 @@
 20:00-9:00</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr">
         <is>
           <t>צרפתי</t>
         </is>
@@ -742,12 +742,12 @@
       </c>
       <c r="G4" s="8" t="inlineStr">
         <is>
-          <t>צרפתי</t>
-        </is>
-      </c>
-      <c r="H4" s="7" t="inlineStr">
-        <is>
           <t>עומר</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>ניר</t>
         </is>
       </c>
     </row>
@@ -796,17 +796,17 @@
       </c>
       <c r="B8" s="15" t="inlineStr">
         <is>
-          <t>ניר: 4</t>
+          <t>ניר: 6</t>
         </is>
       </c>
       <c r="C8" s="15" t="inlineStr">
         <is>
-          <t>משה: 4</t>
+          <t>משה: 3</t>
         </is>
       </c>
       <c r="D8" s="15" t="inlineStr">
         <is>
-          <t>עומר: 5</t>
+          <t>עומר: 7</t>
         </is>
       </c>
       <c r="E8" s="15" t="inlineStr">
@@ -816,7 +816,7 @@
       </c>
       <c r="F8" s="15" t="inlineStr">
         <is>
-          <t>צרפתי: 6</t>
+          <t>צרפתי: 3</t>
         </is>
       </c>
       <c r="G8" s="15" t="inlineStr">
@@ -920,29 +920,29 @@
           <t>עומרי</t>
         </is>
       </c>
-      <c r="D2" s="9" t="inlineStr">
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>צרפתי</t>
+        </is>
+      </c>
+      <c r="E2" s="8" t="inlineStr">
+        <is>
+          <t>עומר</t>
+        </is>
+      </c>
+      <c r="F2" s="8" t="inlineStr">
+        <is>
+          <t>עומר</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>ניר</t>
+        </is>
+      </c>
+      <c r="H2" s="9" t="inlineStr">
         <is>
           <t>משה</t>
-        </is>
-      </c>
-      <c r="E2" s="7" t="inlineStr">
-        <is>
-          <t>עומר</t>
-        </is>
-      </c>
-      <c r="F2" s="8" t="inlineStr">
-        <is>
-          <t>צרפתי</t>
-        </is>
-      </c>
-      <c r="G2" s="7" t="inlineStr">
-        <is>
-          <t>עומר</t>
-        </is>
-      </c>
-      <c r="H2" s="5" t="inlineStr">
-        <is>
-          <t>ניר</t>
         </is>
       </c>
     </row>
@@ -958,7 +958,7 @@
           <t>עומרי</t>
         </is>
       </c>
-      <c r="C3" s="7" t="inlineStr">
+      <c r="C3" s="8" t="inlineStr">
         <is>
           <t>עומר</t>
         </is>
@@ -983,9 +983,9 @@
           <t>אורי הלוי</t>
         </is>
       </c>
-      <c r="H3" s="5" t="inlineStr">
-        <is>
-          <t>ניר</t>
+      <c r="H3" s="9" t="inlineStr">
+        <is>
+          <t>משה</t>
         </is>
       </c>
     </row>
@@ -996,7 +996,7 @@
 20:00-9:00</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr">
         <is>
           <t>צרפתי</t>
         </is>
@@ -1023,12 +1023,12 @@
       </c>
       <c r="G4" s="8" t="inlineStr">
         <is>
-          <t>צרפתי</t>
-        </is>
-      </c>
-      <c r="H4" s="7" t="inlineStr">
-        <is>
           <t>עומר</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>ניר</t>
         </is>
       </c>
     </row>
@@ -1077,12 +1077,12 @@
       </c>
       <c r="B8" s="15" t="inlineStr">
         <is>
-          <t>ניר: 5</t>
+          <t>ניר: 6</t>
         </is>
       </c>
       <c r="C8" s="15" t="inlineStr">
         <is>
-          <t>משה: 4</t>
+          <t>משה: 5</t>
         </is>
       </c>
       <c r="D8" s="15" t="inlineStr">
@@ -1097,7 +1097,7 @@
       </c>
       <c r="F8" s="15" t="inlineStr">
         <is>
-          <t>צרפתי: 5</t>
+          <t>צרפתי: 3</t>
         </is>
       </c>
       <c r="G8" s="15" t="inlineStr">

</xml_diff>

<commit_message>
Fix constraints: צרפתי only Sun night + Tue morning, משה Sat evening only, אורי הלוי Wed only
- צרפתי limited to 2 shifts (צו closes Tue night)
- משה: removed Sat morning, keep only Sat evening
- אורי הלוי: blocked Thu/Fri/Sat (only Wed fixed)
- עומר: fixed Fri night
- ניר: covers Fri morning+evening + Sat morning+night (only available)
- Fixed all gaps in both sheets

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/משמרות_29.3-4.4_v2.xlsx
+++ b/משמרות_29.3-4.4_v2.xlsx
@@ -39,11 +39,11 @@
     </font>
     <font>
       <name val="Arial"/>
+      <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
@@ -90,8 +90,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="0000B0F0"/>
-        <bgColor rgb="0000B0F0"/>
+        <fgColor rgb="00FF00FF"/>
+        <bgColor rgb="00FF00FF"/>
       </patternFill>
     </fill>
     <fill>
@@ -114,8 +114,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FF00FF"/>
-        <bgColor rgb="00FF00FF"/>
+        <fgColor rgb="0000B0F0"/>
+        <bgColor rgb="0000B0F0"/>
       </patternFill>
     </fill>
     <fill>
@@ -160,25 +160,25 @@
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -187,7 +187,7 @@
     <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -631,7 +631,7 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>ניר</t>
+          <t>משה</t>
         </is>
       </c>
       <c r="C2" s="6" t="inlineStr">
@@ -654,7 +654,7 @@
           <t>עומר</t>
         </is>
       </c>
-      <c r="G2" s="5" t="inlineStr">
+      <c r="G2" s="9" t="inlineStr">
         <is>
           <t>ניר</t>
         </is>
@@ -684,7 +684,7 @@
       </c>
       <c r="D3" s="9" t="inlineStr">
         <is>
-          <t>משה</t>
+          <t>ניר</t>
         </is>
       </c>
       <c r="E3" s="8" t="inlineStr">
@@ -697,9 +697,9 @@
           <t>עומרי</t>
         </is>
       </c>
-      <c r="G3" s="10" t="inlineStr">
-        <is>
-          <t>אורי הלוי</t>
+      <c r="G3" s="9" t="inlineStr">
+        <is>
+          <t>ניר</t>
         </is>
       </c>
       <c r="H3" s="10" t="inlineStr">
@@ -722,7 +722,7 @@
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>ניר</t>
+          <t>משה</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
@@ -735,7 +735,7 @@
           <t>אורי הלוי</t>
         </is>
       </c>
-      <c r="F4" s="9" t="inlineStr">
+      <c r="F4" s="5" t="inlineStr">
         <is>
           <t>משה</t>
         </is>
@@ -745,7 +745,7 @@
           <t>עומר</t>
         </is>
       </c>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="H4" s="9" t="inlineStr">
         <is>
           <t>ניר</t>
         </is>
@@ -762,7 +762,7 @@
           <t>ניר</t>
         </is>
       </c>
-      <c r="C6" s="9" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>משה</t>
         </is>
@@ -796,12 +796,12 @@
       </c>
       <c r="B8" s="15" t="inlineStr">
         <is>
-          <t>ניר: 6</t>
+          <t>ניר: 5</t>
         </is>
       </c>
       <c r="C8" s="15" t="inlineStr">
         <is>
-          <t>משה: 3</t>
+          <t>משה: 5</t>
         </is>
       </c>
       <c r="D8" s="15" t="inlineStr">
@@ -821,7 +821,7 @@
       </c>
       <c r="G8" s="15" t="inlineStr">
         <is>
-          <t>אורי הלוי: 4</t>
+          <t>אורי הלוי: 3</t>
         </is>
       </c>
     </row>
@@ -912,37 +912,37 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
+          <t>משה</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>עומרי</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>צרפתי</t>
+        </is>
+      </c>
+      <c r="E2" s="8" t="inlineStr">
+        <is>
+          <t>עומר</t>
+        </is>
+      </c>
+      <c r="F2" s="8" t="inlineStr">
+        <is>
+          <t>עומר</t>
+        </is>
+      </c>
+      <c r="G2" s="9" t="inlineStr">
+        <is>
           <t>ניר</t>
         </is>
       </c>
-      <c r="C2" s="6" t="inlineStr">
-        <is>
-          <t>עומרי</t>
-        </is>
-      </c>
-      <c r="D2" s="7" t="inlineStr">
-        <is>
-          <t>צרפתי</t>
-        </is>
-      </c>
-      <c r="E2" s="8" t="inlineStr">
-        <is>
-          <t>עומר</t>
-        </is>
-      </c>
-      <c r="F2" s="8" t="inlineStr">
-        <is>
-          <t>עומר</t>
-        </is>
-      </c>
-      <c r="G2" s="5" t="inlineStr">
+      <c r="H2" s="9" t="inlineStr">
         <is>
           <t>ניר</t>
-        </is>
-      </c>
-      <c r="H2" s="9" t="inlineStr">
-        <is>
-          <t>משה</t>
         </is>
       </c>
     </row>
@@ -965,7 +965,7 @@
       </c>
       <c r="D3" s="9" t="inlineStr">
         <is>
-          <t>משה</t>
+          <t>ניר</t>
         </is>
       </c>
       <c r="E3" s="10" t="inlineStr">
@@ -978,12 +978,12 @@
           <t>עומרי</t>
         </is>
       </c>
-      <c r="G3" s="10" t="inlineStr">
-        <is>
-          <t>אורי הלוי</t>
-        </is>
-      </c>
-      <c r="H3" s="9" t="inlineStr">
+      <c r="G3" s="9" t="inlineStr">
+        <is>
+          <t>ניר</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>משה</t>
         </is>
@@ -1003,7 +1003,7 @@
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>ניר</t>
+          <t>משה</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
@@ -1016,7 +1016,7 @@
           <t>אורי הלוי</t>
         </is>
       </c>
-      <c r="F4" s="9" t="inlineStr">
+      <c r="F4" s="5" t="inlineStr">
         <is>
           <t>משה</t>
         </is>
@@ -1026,7 +1026,7 @@
           <t>עומר</t>
         </is>
       </c>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="H4" s="9" t="inlineStr">
         <is>
           <t>ניר</t>
         </is>
@@ -1043,7 +1043,7 @@
           <t>ניר</t>
         </is>
       </c>
-      <c r="C6" s="9" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>משה</t>
         </is>
@@ -1082,7 +1082,7 @@
       </c>
       <c r="C8" s="15" t="inlineStr">
         <is>
-          <t>משה: 5</t>
+          <t>משה: 6</t>
         </is>
       </c>
       <c r="D8" s="15" t="inlineStr">
@@ -1102,7 +1102,7 @@
       </c>
       <c r="G8" s="15" t="inlineStr">
         <is>
-          <t>אורי הלוי: 4</t>
+          <t>אורי הלוי: 3</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
משה blocked Sunday, ניר fixed Sunday morning for early-week coverage
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/משמרות_29.3-4.4_v2.xlsx
+++ b/משמרות_29.3-4.4_v2.xlsx
@@ -39,11 +39,11 @@
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
+      <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
@@ -90,8 +90,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FF00FF"/>
-        <bgColor rgb="00FF00FF"/>
+        <fgColor rgb="0000B0F0"/>
+        <bgColor rgb="0000B0F0"/>
       </patternFill>
     </fill>
     <fill>
@@ -114,14 +114,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="0000B0F0"/>
-        <bgColor rgb="0000B0F0"/>
+        <fgColor rgb="00FF6600"/>
+        <bgColor rgb="00FF6600"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FF6600"/>
-        <bgColor rgb="00FF6600"/>
+        <fgColor rgb="00FF00FF"/>
+        <bgColor rgb="00FF00FF"/>
       </patternFill>
     </fill>
   </fills>
@@ -160,25 +160,25 @@
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -187,7 +187,7 @@
     <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -631,7 +631,7 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>משה</t>
+          <t>ניר</t>
         </is>
       </c>
       <c r="C2" s="6" t="inlineStr">
@@ -654,7 +654,7 @@
           <t>עומר</t>
         </is>
       </c>
-      <c r="G2" s="9" t="inlineStr">
+      <c r="G2" s="5" t="inlineStr">
         <is>
           <t>ניר</t>
         </is>
@@ -682,7 +682,7 @@
           <t>עומר</t>
         </is>
       </c>
-      <c r="D3" s="9" t="inlineStr">
+      <c r="D3" s="5" t="inlineStr">
         <is>
           <t>ניר</t>
         </is>
@@ -697,12 +697,12 @@
           <t>עומרי</t>
         </is>
       </c>
-      <c r="G3" s="9" t="inlineStr">
-        <is>
-          <t>ניר</t>
-        </is>
-      </c>
-      <c r="H3" s="10" t="inlineStr">
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>ניר</t>
+        </is>
+      </c>
+      <c r="H3" s="9" t="inlineStr">
         <is>
           <t>אורי הלוי</t>
         </is>
@@ -720,7 +720,7 @@
           <t>צרפתי</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="10" t="inlineStr">
         <is>
           <t>משה</t>
         </is>
@@ -730,12 +730,12 @@
           <t>עומרי</t>
         </is>
       </c>
-      <c r="E4" s="10" t="inlineStr">
+      <c r="E4" s="9" t="inlineStr">
         <is>
           <t>אורי הלוי</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="F4" s="10" t="inlineStr">
         <is>
           <t>משה</t>
         </is>
@@ -745,7 +745,7 @@
           <t>עומר</t>
         </is>
       </c>
-      <c r="H4" s="9" t="inlineStr">
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>ניר</t>
         </is>
@@ -762,7 +762,7 @@
           <t>ניר</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" s="10" t="inlineStr">
         <is>
           <t>משה</t>
         </is>
@@ -782,7 +782,7 @@
           <t>צרפתי</t>
         </is>
       </c>
-      <c r="G6" s="10" t="inlineStr">
+      <c r="G6" s="9" t="inlineStr">
         <is>
           <t>אורי הלוי</t>
         </is>
@@ -796,12 +796,12 @@
       </c>
       <c r="B8" s="15" t="inlineStr">
         <is>
-          <t>ניר: 5</t>
+          <t>ניר: 6</t>
         </is>
       </c>
       <c r="C8" s="15" t="inlineStr">
         <is>
-          <t>משה: 5</t>
+          <t>משה: 4</t>
         </is>
       </c>
       <c r="D8" s="15" t="inlineStr">
@@ -912,7 +912,7 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>משה</t>
+          <t>ניר</t>
         </is>
       </c>
       <c r="C2" s="6" t="inlineStr">
@@ -935,12 +935,12 @@
           <t>עומר</t>
         </is>
       </c>
-      <c r="G2" s="9" t="inlineStr">
-        <is>
-          <t>ניר</t>
-        </is>
-      </c>
-      <c r="H2" s="9" t="inlineStr">
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>ניר</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="inlineStr">
         <is>
           <t>ניר</t>
         </is>
@@ -963,12 +963,12 @@
           <t>עומר</t>
         </is>
       </c>
-      <c r="D3" s="9" t="inlineStr">
-        <is>
-          <t>ניר</t>
-        </is>
-      </c>
-      <c r="E3" s="10" t="inlineStr">
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>ניר</t>
+        </is>
+      </c>
+      <c r="E3" s="9" t="inlineStr">
         <is>
           <t>אורי הלוי</t>
         </is>
@@ -978,12 +978,12 @@
           <t>עומרי</t>
         </is>
       </c>
-      <c r="G3" s="9" t="inlineStr">
-        <is>
-          <t>ניר</t>
-        </is>
-      </c>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>ניר</t>
+        </is>
+      </c>
+      <c r="H3" s="10" t="inlineStr">
         <is>
           <t>משה</t>
         </is>
@@ -1001,7 +1001,7 @@
           <t>צרפתי</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="10" t="inlineStr">
         <is>
           <t>משה</t>
         </is>
@@ -1011,12 +1011,12 @@
           <t>עומרי</t>
         </is>
       </c>
-      <c r="E4" s="10" t="inlineStr">
+      <c r="E4" s="9" t="inlineStr">
         <is>
           <t>אורי הלוי</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="F4" s="10" t="inlineStr">
         <is>
           <t>משה</t>
         </is>
@@ -1026,7 +1026,7 @@
           <t>עומר</t>
         </is>
       </c>
-      <c r="H4" s="9" t="inlineStr">
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>ניר</t>
         </is>
@@ -1043,7 +1043,7 @@
           <t>ניר</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" s="10" t="inlineStr">
         <is>
           <t>משה</t>
         </is>
@@ -1063,7 +1063,7 @@
           <t>צרפתי</t>
         </is>
       </c>
-      <c r="G6" s="10" t="inlineStr">
+      <c r="G6" s="9" t="inlineStr">
         <is>
           <t>אורי הלוי</t>
         </is>
@@ -1077,12 +1077,12 @@
       </c>
       <c r="B8" s="15" t="inlineStr">
         <is>
-          <t>ניר: 6</t>
+          <t>ניר: 7</t>
         </is>
       </c>
       <c r="C8" s="15" t="inlineStr">
         <is>
-          <t>משה: 6</t>
+          <t>משה: 5</t>
         </is>
       </c>
       <c r="D8" s="15" t="inlineStr">

</xml_diff>